<commit_message>
Remove theme font override from review tables
</commit_message>
<xml_diff>
--- a/excel/clinical_logic_review_matrix.v1.xlsx
+++ b/excel/clinical_logic_review_matrix.v1.xlsx
@@ -52,33 +52,37 @@
     </font>
     <font>
       <name val="Times New Roman"/>
+      <family val="1"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Times New Roman"/>
+      <family val="1"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="20"/>
     </font>
     <font>
       <name val="Times New Roman"/>
-      <family val="2"/>
+      <family val="1"/>
       <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <name val="Times New Roman"/>
+      <family val="1"/>
       <i val="1"/>
       <color rgb="0044545B"/>
     </font>
     <font>
       <name val="Times New Roman"/>
+      <family val="1"/>
       <b val="1"/>
       <color rgb="007A2F12"/>
     </font>
     <font>
       <name val="Times New Roman"/>
+      <family val="1"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>

</xml_diff>

<commit_message>
Revise clinical framing and simulation outputs
</commit_message>
<xml_diff>
--- a/excel/clinical_logic_review_matrix.v1.xlsx
+++ b/excel/clinical_logic_review_matrix.v1.xlsx
@@ -11,12 +11,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key Scenarios" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Decisions" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Logic Matrix" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Assumptions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Category Assumptions" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Key Scenarios'!$A$7:$K$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Full Logic Matrix'!$A$7:$M$331</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Risk Assumptions'!$A$7:$E$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Category Assumptions'!$A$7:$E$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -649,24 +649,24 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Cachexia rule</t>
+          <t>Baseline-derived cachexia criteria status</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Yes when loss is &gt;5%; or loss is &gt;2% with BMI &lt;20; or loss is &gt;2% with explicitly documented sarcopenia.</t>
+          <t>Yes when retrospective loss is &gt;5%, or loss is &gt;2% with BMI &lt;20. When loss is &gt;2% and &lt;=5%, BMI is &gt;=20, and the sarcopenia branch is disabled pending a clinical definition, status is unknown rather than no.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Provisional early-risk rule</t>
+          <t>Provisional pre-cachexia candidate</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Yes only when cachexia is excluded, loss is &gt;1% and &lt;=5%, and reduced appetite is yes.</t>
+          <t>Yes only when cachexia criteria are excluded, loss is &gt;1% and &lt;=5%, and baseline reduced appetite is yes.</t>
         </is>
       </c>
     </row>
@@ -702,7 +702,7 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Yes = independently documented; no = assessed and absent; unknown = not assessed or not documented. It is never inferred.</t>
+          <t>Future-use tri-state field pending clinical definition. It is never inferred; the disabled branch can leave criteria unknown, but the recorded baseline value does not decide the v1 criteria or categories.</t>
         </is>
       </c>
     </row>
@@ -721,119 +721,107 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Risk percentages</t>
+          <t>Illustrative categories</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Risk Assumptions contains illustrative simulation terms only. They are not calibrated probabilities or validated clinical effects.</t>
+          <t>Category Assumptions contains internal simulation terms only. Clinical-facing outputs are ordinal low, moderate, or high, or withheld. Target outcome is not defined pending clinical review.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Current status</t>
+          <t>Early-rule limitations</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>All rules remain pending clinical review. Recorded feedback documents the review outcome but does not validate the prototype.</t>
+          <t>The &gt;1% lower bound has no consensus basis and is editable; &lt;=5% is consensus-aligned; binary appetite is a POC simplification.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="8" t="n"/>
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Population status</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Eligibility and inclusion criteria are not defined. Cancer labels are synthetic adult solid-tumour stratifiers pending review.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Full-matrix output summary</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="n"/>
+          <t>Fearon citation</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Fearon et al. 2011, Lancet Oncology 12(5):489-495, DOI 10.1016/S1470-2045(10)70218-7. The &gt;5% branch is retrospective over the past 6 months.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Cachexia</t>
+          <t>Pre-cachexia citation</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Early-risk pattern</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>Case count</t>
+          <t>Muscaritoli et al. 2010, Clinical Nutrition 29(2):154-159, DOI 10.1016/j.clnu.2009.12.004. &lt;=5% is consensus-aligned; this POC's &gt;1% lower bound is not.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Current status</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="n">
-        <v>136</v>
+          <t>All rules remain pending clinical review. Recorded feedback documents the review outcome but does not validate the prototype.</t>
+        </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="n">
-        <v>28</v>
-      </c>
+      <c r="B24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="n">
-        <v>28</v>
-      </c>
+          <t>Full-matrix output summary</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>Cachexia</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="n">
-        <v>60</v>
+          <t>Early-risk pattern</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Case count</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -842,7 +830,67 @@
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>72</v>
+        <v>132</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -930,7 +978,7 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>Cachexia result</t>
+          <t>Baseline cachexia criteria status</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
@@ -940,7 +988,7 @@
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>Early-risk result</t>
+          <t>Provisional candidate status</t>
         </is>
       </c>
       <c r="I7" s="9" t="inlineStr">
@@ -1280,7 +1328,7 @@
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Loss over 2% with sarcopenia</t>
+          <t>Loss over 2%; future-use sarcopenia yes</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1305,22 +1353,22 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>Weight loss is &gt;2% and sarcopenia is documented.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>Cachexia criteria take precedence.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="J14" s="10" t="inlineStr">
@@ -1333,7 +1381,7 @@
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Loss over 2%; sarcopenia unknown</t>
+          <t>Loss over 2%; future-use sarcopenia unknown</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
@@ -1363,7 +1411,7 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Not evaluable because sarcopenia are unknown.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
@@ -1411,22 +1459,22 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>BMI and sarcopenia conditional branches are refuted.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>Limited loss and reduced appetite are both present.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="J16" s="10" t="inlineStr">
@@ -1575,7 +1623,7 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Not evaluable because BMI are unknown.</t>
+          <t>Not evaluable because BMI and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
@@ -1640,7 +1688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1779,12 +1827,12 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Should documented sarcopenia identify cachexia when weight loss is greater than 2%?</t>
+          <t>What future evidence and definition should be required before enabling a sarcopenia branch?</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Weight loss &gt;2% and documented sarcopenia</t>
+          <t>Future-use tri-state field; branch disabled in v1</t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr">
@@ -1831,12 +1879,12 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Is the proposed early-risk weight-loss interval appropriate?</t>
+          <t>Is an editable &gt;1% lower bound acceptable despite having no consensus basis?</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Weight loss &gt;1% and &lt;=5%, after cachexia is excluded</t>
+          <t>Weight loss &gt;1%; no consensus basis</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">
@@ -1857,12 +1905,12 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Should reduced appetite be required for the proposed early-risk pattern?</t>
+          <t>Is the consensus-aligned &lt;=5% upper bound and binary appetite simplification acceptable for the provisional candidate rule?</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Reduced appetite = yes</t>
+          <t>&lt;=5% and baseline reduced appetite=yes</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -1883,12 +1931,12 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>What evidence should count as documented sarcopenia, and can baseline evidence be carried into future outcome labels?</t>
+          <t>What evidence should count as documented sarcopenia before any future branch is enabled?</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Explicit yes/no/unknown evidence; provisional baseline carry-forward</t>
+          <t>Explicit future-use yes/no/unknown; never inferred; unused in v1</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr">
@@ -1935,12 +1983,12 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Should the illustrative risk percentages remain in the demonstrator?</t>
+          <t>What target outcome or estimand should the clinical team define before ordinal categories can be interpreted?</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Configured simulation coefficients and multipliers; not clinically validated</t>
+          <t>Target outcome is not defined pending clinical review; low/moderate/high categories are illustrative only</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
@@ -1952,6 +2000,84 @@
       <c r="F16" s="12" t="n"/>
       <c r="G16" s="11" t="n"/>
       <c r="H16" s="11" t="n"/>
+    </row>
+    <row r="17" ht="44" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>MATRIX-010</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>What eligibility and inclusion criteria define the intended population?</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Not yet defined; synthetic adult solid-tumour stratifiers only</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="n"/>
+      <c r="F17" s="12" t="n"/>
+      <c r="G17" s="11" t="n"/>
+      <c r="H17" s="11" t="n"/>
+    </row>
+    <row r="18" ht="44" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>MATRIX-011</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Are dated follow-up appetite observations appropriate evidence for future provisional labels?</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Baseline appetite is never carried forward</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="n"/>
+      <c r="F18" s="12" t="n"/>
+      <c r="G18" s="11" t="n"/>
+      <c r="H18" s="11" t="n"/>
+    </row>
+    <row r="19" ht="44" customHeight="1">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>MATRIX-012</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Are the 3-month threshold outcome and prospective 6-month research endpoint framed clearly enough?</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Neither is a Fearon classification; the 6m endpoint matches the window length but looks forward and is not a diagnosis</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="n"/>
+      <c r="F19" s="12" t="n"/>
+      <c r="G19" s="11" t="n"/>
+      <c r="H19" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1960,7 +2086,7 @@
     <mergeCell ref="A2:P2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="D8:D16" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" error="Select pending, approved, rejected, or revision_requested." promptTitle="Decision status" prompt="Available values: pending, approved, rejected, or revision_requested." type="list" errorStyle="stop">
+    <dataValidation sqref="D8:D19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" error="Select pending, approved, rejected, or revision_requested." promptTitle="Decision status" prompt="Available values: pending, approved, rejected, or revision_requested." type="list" errorStyle="stop">
       <formula1>"pending,approved,rejected,revision_requested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2050,7 +2176,7 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>Cachexia result</t>
+          <t>Baseline cachexia criteria status</t>
         </is>
       </c>
       <c r="H7" s="9" t="inlineStr">
@@ -2060,7 +2186,7 @@
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>Early-risk result</t>
+          <t>Provisional candidate status</t>
         </is>
       </c>
       <c r="J7" s="9" t="inlineStr">
@@ -15183,22 +15309,22 @@
       </c>
       <c r="G224" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H224" s="7" t="inlineStr">
         <is>
-          <t>Weight loss is &gt;2% and sarcopenia is documented.</t>
+          <t>Not evaluable because BMI and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I224" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J224" s="7" t="inlineStr">
         <is>
-          <t>Cachexia criteria take precedence.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K224" s="6" t="inlineStr">
@@ -15244,22 +15370,22 @@
       </c>
       <c r="G225" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H225" s="7" t="inlineStr">
         <is>
-          <t>Weight loss is &gt;2% and sarcopenia is documented.</t>
+          <t>Not evaluable because BMI and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I225" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J225" s="7" t="inlineStr">
         <is>
-          <t>Cachexia criteria take precedence.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K225" s="6" t="inlineStr">
@@ -15305,22 +15431,22 @@
       </c>
       <c r="G226" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H226" s="7" t="inlineStr">
         <is>
-          <t>Weight loss is &gt;2% and sarcopenia is documented.</t>
+          <t>Not evaluable because BMI and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I226" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J226" s="7" t="inlineStr">
         <is>
-          <t>Cachexia criteria take precedence.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K226" s="6" t="inlineStr">
@@ -15371,7 +15497,7 @@
       </c>
       <c r="H227" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because BMI are unknown.</t>
+          <t>Not evaluable because BMI and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I227" s="6" t="inlineStr">
@@ -15432,7 +15558,7 @@
       </c>
       <c r="H228" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because BMI are unknown.</t>
+          <t>Not evaluable because BMI and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I228" s="6" t="inlineStr">
@@ -15493,7 +15619,7 @@
       </c>
       <c r="H229" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because BMI are unknown.</t>
+          <t>Not evaluable because BMI and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I229" s="6" t="inlineStr">
@@ -15554,7 +15680,7 @@
       </c>
       <c r="H230" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because BMI and sarcopenia are unknown.</t>
+          <t>Not evaluable because BMI and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I230" s="6" t="inlineStr">
@@ -15615,7 +15741,7 @@
       </c>
       <c r="H231" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because BMI and sarcopenia are unknown.</t>
+          <t>Not evaluable because BMI and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I231" s="6" t="inlineStr">
@@ -15676,7 +15802,7 @@
       </c>
       <c r="H232" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because BMI and sarcopenia are unknown.</t>
+          <t>Not evaluable because BMI and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I232" s="6" t="inlineStr">
@@ -16281,22 +16407,22 @@
       </c>
       <c r="G242" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H242" s="7" t="inlineStr">
         <is>
-          <t>Weight loss is &gt;2% and sarcopenia is documented.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I242" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J242" s="7" t="inlineStr">
         <is>
-          <t>Cachexia criteria take precedence.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K242" s="6" t="inlineStr">
@@ -16342,22 +16468,22 @@
       </c>
       <c r="G243" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H243" s="7" t="inlineStr">
         <is>
-          <t>Weight loss is &gt;2% and sarcopenia is documented.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I243" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J243" s="7" t="inlineStr">
         <is>
-          <t>Cachexia criteria take precedence.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K243" s="6" t="inlineStr">
@@ -16403,22 +16529,22 @@
       </c>
       <c r="G244" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H244" s="7" t="inlineStr">
         <is>
-          <t>Weight loss is &gt;2% and sarcopenia is documented.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I244" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J244" s="7" t="inlineStr">
         <is>
-          <t>Cachexia criteria take precedence.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K244" s="6" t="inlineStr">
@@ -16464,22 +16590,22 @@
       </c>
       <c r="G245" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H245" s="7" t="inlineStr">
         <is>
-          <t>BMI and sarcopenia conditional branches are refuted.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I245" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J245" s="7" t="inlineStr">
         <is>
-          <t>Limited loss and reduced appetite are both present.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K245" s="6" t="inlineStr">
@@ -16525,22 +16651,22 @@
       </c>
       <c r="G246" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H246" s="7" t="inlineStr">
         <is>
-          <t>BMI and sarcopenia conditional branches are refuted.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I246" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J246" s="7" t="inlineStr">
         <is>
-          <t>Reduced appetite is explicitly absent.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K246" s="6" t="inlineStr">
@@ -16586,12 +16712,12 @@
       </c>
       <c r="G247" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H247" s="7" t="inlineStr">
         <is>
-          <t>BMI and sarcopenia conditional branches are refuted.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I247" s="6" t="inlineStr">
@@ -16601,7 +16727,7 @@
       </c>
       <c r="J247" s="7" t="inlineStr">
         <is>
-          <t>Reduced appetite is unknown.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K247" s="6" t="inlineStr">
@@ -16652,7 +16778,7 @@
       </c>
       <c r="H248" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because sarcopenia are unknown.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I248" s="6" t="inlineStr">
@@ -16713,7 +16839,7 @@
       </c>
       <c r="H249" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because sarcopenia are unknown.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I249" s="6" t="inlineStr">
@@ -16774,7 +16900,7 @@
       </c>
       <c r="H250" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because sarcopenia are unknown.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I250" s="6" t="inlineStr">
@@ -16830,22 +16956,22 @@
       </c>
       <c r="G251" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H251" s="7" t="inlineStr">
         <is>
-          <t>Weight loss is &gt;2% and sarcopenia is documented.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I251" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J251" s="7" t="inlineStr">
         <is>
-          <t>Cachexia criteria take precedence.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K251" s="6" t="inlineStr">
@@ -16891,22 +17017,22 @@
       </c>
       <c r="G252" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H252" s="7" t="inlineStr">
         <is>
-          <t>Weight loss is &gt;2% and sarcopenia is documented.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I252" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J252" s="7" t="inlineStr">
         <is>
-          <t>Cachexia criteria take precedence.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K252" s="6" t="inlineStr">
@@ -16952,22 +17078,22 @@
       </c>
       <c r="G253" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H253" s="7" t="inlineStr">
         <is>
-          <t>Weight loss is &gt;2% and sarcopenia is documented.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I253" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J253" s="7" t="inlineStr">
         <is>
-          <t>Cachexia criteria take precedence.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K253" s="6" t="inlineStr">
@@ -17013,22 +17139,22 @@
       </c>
       <c r="G254" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H254" s="7" t="inlineStr">
         <is>
-          <t>BMI and sarcopenia conditional branches are refuted.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I254" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J254" s="7" t="inlineStr">
         <is>
-          <t>Limited loss and reduced appetite are both present.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K254" s="6" t="inlineStr">
@@ -17074,22 +17200,22 @@
       </c>
       <c r="G255" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H255" s="7" t="inlineStr">
         <is>
-          <t>BMI and sarcopenia conditional branches are refuted.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I255" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J255" s="7" t="inlineStr">
         <is>
-          <t>Reduced appetite is explicitly absent.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K255" s="6" t="inlineStr">
@@ -17135,12 +17261,12 @@
       </c>
       <c r="G256" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H256" s="7" t="inlineStr">
         <is>
-          <t>BMI and sarcopenia conditional branches are refuted.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I256" s="6" t="inlineStr">
@@ -17150,7 +17276,7 @@
       </c>
       <c r="J256" s="7" t="inlineStr">
         <is>
-          <t>Reduced appetite is unknown.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K256" s="6" t="inlineStr">
@@ -17201,7 +17327,7 @@
       </c>
       <c r="H257" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because sarcopenia are unknown.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I257" s="6" t="inlineStr">
@@ -17262,7 +17388,7 @@
       </c>
       <c r="H258" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because sarcopenia are unknown.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I258" s="6" t="inlineStr">
@@ -17323,7 +17449,7 @@
       </c>
       <c r="H259" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because sarcopenia are unknown.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I259" s="6" t="inlineStr">
@@ -17379,22 +17505,22 @@
       </c>
       <c r="G260" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H260" s="7" t="inlineStr">
         <is>
-          <t>Weight loss is &gt;2% and sarcopenia is documented.</t>
+          <t>Not evaluable because BMI and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I260" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J260" s="7" t="inlineStr">
         <is>
-          <t>Cachexia criteria take precedence.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K260" s="6" t="inlineStr">
@@ -17440,22 +17566,22 @@
       </c>
       <c r="G261" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H261" s="7" t="inlineStr">
         <is>
-          <t>Weight loss is &gt;2% and sarcopenia is documented.</t>
+          <t>Not evaluable because BMI and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I261" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J261" s="7" t="inlineStr">
         <is>
-          <t>Cachexia criteria take precedence.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K261" s="6" t="inlineStr">
@@ -17501,22 +17627,22 @@
       </c>
       <c r="G262" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H262" s="7" t="inlineStr">
         <is>
-          <t>Weight loss is &gt;2% and sarcopenia is documented.</t>
+          <t>Not evaluable because BMI and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I262" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J262" s="7" t="inlineStr">
         <is>
-          <t>Cachexia criteria take precedence.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K262" s="6" t="inlineStr">
@@ -17567,7 +17693,7 @@
       </c>
       <c r="H263" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because BMI are unknown.</t>
+          <t>Not evaluable because BMI and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I263" s="6" t="inlineStr">
@@ -17628,7 +17754,7 @@
       </c>
       <c r="H264" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because BMI are unknown.</t>
+          <t>Not evaluable because BMI and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I264" s="6" t="inlineStr">
@@ -17689,7 +17815,7 @@
       </c>
       <c r="H265" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because BMI are unknown.</t>
+          <t>Not evaluable because BMI and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I265" s="6" t="inlineStr">
@@ -17750,7 +17876,7 @@
       </c>
       <c r="H266" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because BMI and sarcopenia are unknown.</t>
+          <t>Not evaluable because BMI and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I266" s="6" t="inlineStr">
@@ -17811,7 +17937,7 @@
       </c>
       <c r="H267" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because BMI and sarcopenia are unknown.</t>
+          <t>Not evaluable because BMI and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I267" s="6" t="inlineStr">
@@ -17872,7 +17998,7 @@
       </c>
       <c r="H268" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because BMI and sarcopenia are unknown.</t>
+          <t>Not evaluable because BMI and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I268" s="6" t="inlineStr">
@@ -18477,22 +18603,22 @@
       </c>
       <c r="G278" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H278" s="7" t="inlineStr">
         <is>
-          <t>Weight loss is &gt;2% and sarcopenia is documented.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I278" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J278" s="7" t="inlineStr">
         <is>
-          <t>Cachexia criteria take precedence.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K278" s="6" t="inlineStr">
@@ -18538,22 +18664,22 @@
       </c>
       <c r="G279" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H279" s="7" t="inlineStr">
         <is>
-          <t>Weight loss is &gt;2% and sarcopenia is documented.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I279" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J279" s="7" t="inlineStr">
         <is>
-          <t>Cachexia criteria take precedence.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K279" s="6" t="inlineStr">
@@ -18599,22 +18725,22 @@
       </c>
       <c r="G280" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H280" s="7" t="inlineStr">
         <is>
-          <t>Weight loss is &gt;2% and sarcopenia is documented.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I280" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J280" s="7" t="inlineStr">
         <is>
-          <t>Cachexia criteria take precedence.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K280" s="6" t="inlineStr">
@@ -18660,22 +18786,22 @@
       </c>
       <c r="G281" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H281" s="7" t="inlineStr">
         <is>
-          <t>BMI and sarcopenia conditional branches are refuted.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I281" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J281" s="7" t="inlineStr">
         <is>
-          <t>Limited loss and reduced appetite are both present.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K281" s="6" t="inlineStr">
@@ -18721,22 +18847,22 @@
       </c>
       <c r="G282" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H282" s="7" t="inlineStr">
         <is>
-          <t>BMI and sarcopenia conditional branches are refuted.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I282" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J282" s="7" t="inlineStr">
         <is>
-          <t>Reduced appetite is explicitly absent.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K282" s="6" t="inlineStr">
@@ -18782,12 +18908,12 @@
       </c>
       <c r="G283" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H283" s="7" t="inlineStr">
         <is>
-          <t>BMI and sarcopenia conditional branches are refuted.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I283" s="6" t="inlineStr">
@@ -18797,7 +18923,7 @@
       </c>
       <c r="J283" s="7" t="inlineStr">
         <is>
-          <t>Reduced appetite is unknown.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K283" s="6" t="inlineStr">
@@ -18848,7 +18974,7 @@
       </c>
       <c r="H284" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because sarcopenia are unknown.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I284" s="6" t="inlineStr">
@@ -18909,7 +19035,7 @@
       </c>
       <c r="H285" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because sarcopenia are unknown.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I285" s="6" t="inlineStr">
@@ -18970,7 +19096,7 @@
       </c>
       <c r="H286" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because sarcopenia are unknown.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I286" s="6" t="inlineStr">
@@ -19026,22 +19152,22 @@
       </c>
       <c r="G287" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H287" s="7" t="inlineStr">
         <is>
-          <t>Weight loss is &gt;2% and sarcopenia is documented.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I287" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J287" s="7" t="inlineStr">
         <is>
-          <t>Cachexia criteria take precedence.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K287" s="6" t="inlineStr">
@@ -19087,22 +19213,22 @@
       </c>
       <c r="G288" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H288" s="7" t="inlineStr">
         <is>
-          <t>Weight loss is &gt;2% and sarcopenia is documented.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I288" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J288" s="7" t="inlineStr">
         <is>
-          <t>Cachexia criteria take precedence.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K288" s="6" t="inlineStr">
@@ -19148,22 +19274,22 @@
       </c>
       <c r="G289" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H289" s="7" t="inlineStr">
         <is>
-          <t>Weight loss is &gt;2% and sarcopenia is documented.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I289" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J289" s="7" t="inlineStr">
         <is>
-          <t>Cachexia criteria take precedence.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K289" s="6" t="inlineStr">
@@ -19209,22 +19335,22 @@
       </c>
       <c r="G290" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H290" s="7" t="inlineStr">
         <is>
-          <t>BMI and sarcopenia conditional branches are refuted.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I290" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J290" s="7" t="inlineStr">
         <is>
-          <t>Limited loss and reduced appetite are both present.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K290" s="6" t="inlineStr">
@@ -19270,22 +19396,22 @@
       </c>
       <c r="G291" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H291" s="7" t="inlineStr">
         <is>
-          <t>BMI and sarcopenia conditional branches are refuted.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I291" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J291" s="7" t="inlineStr">
         <is>
-          <t>Reduced appetite is explicitly absent.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K291" s="6" t="inlineStr">
@@ -19331,12 +19457,12 @@
       </c>
       <c r="G292" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H292" s="7" t="inlineStr">
         <is>
-          <t>BMI and sarcopenia conditional branches are refuted.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I292" s="6" t="inlineStr">
@@ -19346,7 +19472,7 @@
       </c>
       <c r="J292" s="7" t="inlineStr">
         <is>
-          <t>Reduced appetite is unknown.</t>
+          <t>Cachexia has not been excluded.</t>
         </is>
       </c>
       <c r="K292" s="6" t="inlineStr">
@@ -19397,7 +19523,7 @@
       </c>
       <c r="H293" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because sarcopenia are unknown.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I293" s="6" t="inlineStr">
@@ -19458,7 +19584,7 @@
       </c>
       <c r="H294" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because sarcopenia are unknown.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I294" s="6" t="inlineStr">
@@ -19519,7 +19645,7 @@
       </c>
       <c r="H295" s="7" t="inlineStr">
         <is>
-          <t>Not evaluable because sarcopenia are unknown.</t>
+          <t>Not evaluable in v1 because the BMI branch is not met and the sarcopenia branch is disabled pending a clinical definition.</t>
         </is>
       </c>
       <c r="I295" s="6" t="inlineStr">
@@ -21785,7 +21911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P57"/>
+  <dimension ref="A1:P62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -21798,14 +21924,14 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Illustrative risk-score terms</t>
+          <t>Illustrative simulation category assumptions</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Simulation assumptions only; these values are not validated clinical effects.</t>
+          <t>Internal arithmetic assumptions only; clinical-facing outputs are ordinal categories.</t>
         </is>
       </c>
     </row>
@@ -21854,45 +21980,39 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>intercept</t>
+          <t>target_outcome</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>-2</v>
+          <t>not_defined_pending_clinical_review</t>
+        </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>Target outcome is not defined pending clinical review; the category is illustrative only.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>three_month</t>
+          <t>six_month</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>age_over_55</t>
+          <t>target_outcome</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>0.25</v>
+          <t>not_defined_pending_clinical_review</t>
+        </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>Target outcome is not defined pending clinical review; the category is illustrative only.</t>
         </is>
       </c>
     </row>
@@ -21904,7 +22024,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>baseline_weight_loss_per_percent</t>
+          <t>intercept</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -21913,11 +22033,11 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.13</v>
+        <v>-2</v>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -21929,7 +22049,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>low_bmi_under_20</t>
+          <t>age_over_55</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -21938,11 +22058,11 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.45</v>
+        <v>0.25</v>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -21954,7 +22074,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>cancer_type_multiplier</t>
+          <t>baseline_weight_loss_per_percent</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -21963,11 +22083,11 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>1</v>
+        <v>0.13</v>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -21979,20 +22099,20 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>stage</t>
+          <t>low_bmi_under_20</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>all</t>
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22004,20 +22124,20 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>stage</t>
+          <t>cancer_type_multiplier</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>all</t>
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22034,15 +22154,15 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22059,15 +22179,15 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>II</t>
         </is>
       </c>
       <c r="D16" s="6" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22084,15 +22204,15 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>III</t>
         </is>
       </c>
       <c r="D17" s="6" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22104,20 +22224,20 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>ecog</t>
+          <t>stage</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>IV</t>
         </is>
       </c>
       <c r="D18" s="6" t="n">
-        <v>-0.3</v>
+        <v>1</v>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22129,12 +22249,12 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>ecog</t>
+          <t>stage</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="D19" s="6" t="n">
@@ -22142,7 +22262,7 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22159,15 +22279,15 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>0.35</v>
+        <v>-0.3</v>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22184,15 +22304,15 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D21" s="6" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22209,15 +22329,15 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>1</v>
+        <v>0.35</v>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22234,15 +22354,15 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22254,20 +22374,20 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>appetite</t>
+          <t>ecog</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22279,12 +22399,12 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>appetite</t>
+          <t>ecog</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="D25" s="6" t="n">
@@ -22292,7 +22412,7 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22309,65 +22429,65 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>0.15</v>
+        <v>0.75</v>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>six_month</t>
+          <t>three_month</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>intercept</t>
+          <t>appetite</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>no</t>
         </is>
       </c>
       <c r="D27" s="6" t="n">
-        <v>-1.45</v>
+        <v>0</v>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>six_month</t>
+          <t>three_month</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>age_over_55</t>
+          <t>appetite</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="D28" s="6" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22379,7 +22499,7 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>baseline_weight_loss_per_percent</t>
+          <t>intercept</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -22388,11 +22508,11 @@
         </is>
       </c>
       <c r="D29" s="6" t="n">
-        <v>0.15</v>
+        <v>-1.45</v>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22404,7 +22524,7 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>low_bmi_under_20</t>
+          <t>age_over_55</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -22413,11 +22533,11 @@
         </is>
       </c>
       <c r="D30" s="6" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22429,7 +22549,7 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>cancer_type_multiplier</t>
+          <t>baseline_weight_loss_per_percent</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -22438,11 +22558,11 @@
         </is>
       </c>
       <c r="D31" s="6" t="n">
-        <v>1</v>
+        <v>0.15</v>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22454,20 +22574,20 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>stage</t>
+          <t>low_bmi_under_20</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>all</t>
         </is>
       </c>
       <c r="D32" s="6" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22479,20 +22599,20 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>stage</t>
+          <t>cancer_type_multiplier</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>all</t>
         </is>
       </c>
       <c r="D33" s="6" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22509,15 +22629,15 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D34" s="6" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22534,15 +22654,15 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>IV</t>
+          <t>II</t>
         </is>
       </c>
       <c r="D35" s="6" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22559,15 +22679,15 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>III</t>
         </is>
       </c>
       <c r="D36" s="6" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22579,20 +22699,20 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>ecog</t>
+          <t>stage</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>IV</t>
         </is>
       </c>
       <c r="D37" s="6" t="n">
-        <v>-0.25</v>
+        <v>1</v>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22604,12 +22724,12 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>ecog</t>
+          <t>stage</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="D38" s="6" t="n">
@@ -22617,7 +22737,7 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22634,15 +22754,15 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D39" s="6" t="n">
-        <v>0.4</v>
+        <v>-0.25</v>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22659,15 +22779,15 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D40" s="6" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22684,15 +22804,15 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D41" s="6" t="n">
-        <v>1.1</v>
+        <v>0.4</v>
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22709,15 +22829,15 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D42" s="6" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22729,20 +22849,20 @@
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>appetite</t>
+          <t>ecog</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D43" s="6" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22754,12 +22874,12 @@
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>appetite</t>
+          <t>ecog</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="D44" s="6" t="n">
@@ -22767,7 +22887,7 @@
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
+          <t>internal simulation assumption; not clinically validated</t>
         </is>
       </c>
     </row>
@@ -22784,150 +22904,124 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="D45" s="6" t="n">
-        <v>0.15</v>
+        <v>0.8</v>
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>simulation assumption; not clinically validated</t>
-        </is>
-      </c>
-    </row>
-    <row r="46"/>
+          <t>internal simulation assumption; not clinically validated</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>six_month</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>appetite</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>internal simulation assumption; not clinically validated</t>
+        </is>
+      </c>
+    </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>six_month</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>cancer risk multiplier</t>
+          <t>appetite</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Cancer type</t>
-        </is>
-      </c>
-      <c r="D47" s="6" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="n">
+        <v>0.15</v>
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="6" t="inlineStr">
-        <is>
-          <t>both</t>
-        </is>
-      </c>
-      <c r="B48" s="6" t="inlineStr">
-        <is>
-          <t>cancer risk multiplier</t>
-        </is>
-      </c>
-      <c r="C48" s="6" t="inlineStr">
-        <is>
-          <t>lung</t>
-        </is>
-      </c>
-      <c r="D48" s="6" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="E48" s="6" t="inlineStr">
-        <is>
-          <t>supplied illustrative assumption; not a relative risk</t>
-        </is>
-      </c>
-    </row>
+          <t>internal simulation assumption; not clinically validated</t>
+        </is>
+      </c>
+    </row>
+    <row r="48"/>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>both</t>
+          <t>Shared</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>cancer risk multiplier</t>
+          <t>category boundary</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>colorectal</t>
+          <t>low upper exclusive</t>
         </is>
       </c>
       <c r="D49" s="6" t="n">
-        <v>1.3</v>
+        <v>-0.8472978603872036</v>
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>supplied illustrative assumption; not a relative risk</t>
+          <t>internal simulation assumption; not a clinical threshold</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>both</t>
+          <t>Shared</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>cancer risk multiplier</t>
+          <t>category boundary</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>oesophageal</t>
+          <t>high lower inclusive</t>
         </is>
       </c>
       <c r="D50" s="6" t="n">
-        <v>1.8</v>
+        <v>0.4054651081081642</v>
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>supplied illustrative assumption; not a relative risk</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="6" t="inlineStr">
-        <is>
-          <t>both</t>
-        </is>
-      </c>
-      <c r="B51" s="6" t="inlineStr">
-        <is>
-          <t>cancer risk multiplier</t>
-        </is>
-      </c>
-      <c r="C51" s="6" t="inlineStr">
-        <is>
-          <t>gastric</t>
-        </is>
-      </c>
-      <c r="D51" s="6" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="E51" s="6" t="inlineStr">
-        <is>
-          <t>supplied illustrative assumption; not a relative risk</t>
-        </is>
-      </c>
-    </row>
+          <t>internal simulation assumption; not a clinical threshold</t>
+        </is>
+      </c>
+    </row>
+    <row r="51"/>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>both</t>
+          <t>Shared</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
@@ -22937,15 +23031,17 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>pancreatic</t>
-        </is>
-      </c>
-      <c r="D52" s="6" t="n">
-        <v>2</v>
+          <t>Cancer type</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>supplied illustrative assumption; not a relative risk</t>
+          <t>Status</t>
         </is>
       </c>
     </row>
@@ -22962,15 +23058,15 @@
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>hepatobiliary</t>
+          <t>lung</t>
         </is>
       </c>
       <c r="D53" s="6" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>supplied illustrative assumption; not a relative risk</t>
+          <t>supplied illustrative assumption; not a clinical effect</t>
         </is>
       </c>
     </row>
@@ -22987,15 +23083,15 @@
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>head and neck</t>
+          <t>colorectal</t>
         </is>
       </c>
       <c r="D54" s="6" t="n">
-        <v>1.6</v>
+        <v>1.3</v>
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>supplied illustrative assumption; not a relative risk</t>
+          <t>supplied illustrative assumption; not a clinical effect</t>
         </is>
       </c>
     </row>
@@ -23012,15 +23108,15 @@
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>breast</t>
+          <t>oesophageal</t>
         </is>
       </c>
       <c r="D55" s="6" t="n">
-        <v>1</v>
+        <v>1.8</v>
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t>supplied illustrative assumption; not a relative risk</t>
+          <t>supplied illustrative assumption; not a clinical effect</t>
         </is>
       </c>
     </row>
@@ -23037,15 +23133,15 @@
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>prostate</t>
+          <t>gastric</t>
         </is>
       </c>
       <c r="D56" s="6" t="n">
-        <v>1</v>
+        <v>1.8</v>
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>supplied illustrative assumption; not a relative risk</t>
+          <t>supplied illustrative assumption; not a clinical effect</t>
         </is>
       </c>
     </row>
@@ -23062,20 +23158,145 @@
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
+          <t>pancreatic</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>supplied illustrative assumption; not a clinical effect</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>cancer risk multiplier</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>hepatobiliary</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>supplied illustrative assumption; not a clinical effect</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>cancer risk multiplier</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>head and neck</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>supplied illustrative assumption; not a clinical effect</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>cancer risk multiplier</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>breast</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>supplied illustrative assumption; not a clinical effect</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>cancer risk multiplier</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>prostate</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" s="6" t="inlineStr">
+        <is>
+          <t>supplied illustrative assumption; not a clinical effect</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>cancer risk multiplier</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
           <t>other solid tumour</t>
         </is>
       </c>
-      <c r="D57" s="6" t="n">
+      <c r="D62" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E57" s="6" t="inlineStr">
-        <is>
-          <t>supplied illustrative assumption; not a relative risk</t>
+      <c r="E62" s="6" t="inlineStr">
+        <is>
+          <t>supplied illustrative assumption; not a clinical effect</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A7:E57"/>
+  <autoFilter ref="A7:E62"/>
   <mergeCells count="3">
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A4:P5"/>

</xml_diff>